<commit_message>
Recover pre-clean working tree snapshot
</commit_message>
<xml_diff>
--- a/readme/武器、忍術.xlsx
+++ b/readme/武器、忍術.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lane6\Documents\Codex\忍豆風雲2單機版\readme\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80575969-A5AA-4B93-AA90-ED60B173600E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C72019-3D4C-463C-B688-5E77A854DECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="武器" sheetId="1" r:id="rId1"/>
     <sheet name="忍術" sheetId="2" r:id="rId2"/>
+    <sheet name="rest" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">忍術!$H$3:$M$38</definedName>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="119">
   <si>
     <t>武器</t>
   </si>
@@ -58693,4 +58694,82 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07879590-0CB9-4689-88B8-4F92C3EF4FD6}">
+  <dimension ref="E1:I4"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <sheetData>
+    <row r="1" spans="5:9">
+      <c r="E1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="5:9" ht="37.5">
+      <c r="E2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4">
+        <v>100</v>
+      </c>
+      <c r="H2" s="4">
+        <v>1</v>
+      </c>
+      <c r="I2" s="5">
+        <f>G2/H2</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="5:9" ht="37.5">
+      <c r="E3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G3" s="6">
+        <v>70</v>
+      </c>
+      <c r="H3" s="6">
+        <v>1</v>
+      </c>
+      <c r="I3" s="7">
+        <f>G3/H3</f>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="5:9" ht="37.5">
+      <c r="E4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4">
+        <v>25</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="I4" s="5">
+        <f>G4/H4</f>
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>